<commit_message>
made new changes for the new excel file since its contains new columns
</commit_message>
<xml_diff>
--- a/tests/fixtures/vizient_sample.xlsx
+++ b/tests/fixtures/vizient_sample.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Duplicate Vizent for Data Manip" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,1128 +413,1082 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Nurse ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Organization</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Cohort Date</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Deid_Names</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Employment Start Date</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Type of Unit</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Age</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Gender</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Nursing Degree Received</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>GPA</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Employment Status</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Previous health care work experience</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Leave</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Type of Leave</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Termination</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Termination Date</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Tenure</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Termination Reason</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Termination Updated By</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>organization</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>cohort date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>nurse id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>deid_names</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>employment start date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>type of unit</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>education</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>nursing degree received</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>gpa</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>employment status</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>previous health care work experience</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>leave</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>type of leave</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>termination</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>termination date</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>tenure</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>termination reason</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>termination updated by</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>education (cleaned)</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>id</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N001	</t>
+          <t>Emory University Hospital</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emory University Hospital Midtown	</t>
+          <t xml:space="preserve">	08/28/2023</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">08/28/2023	</t>
+          <t xml:space="preserve">	N001</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nurse A	</t>
+          <t>99001</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">08/04/2023	</t>
+          <t>08/01/2023</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oncology	</t>
+          <t>Med/Surg</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">28	</t>
+          <t>28</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Female	</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emory University	</t>
+          <t>Emory University</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSN	</t>
+          <t>BSN</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.5 and above	</t>
+          <t>3.5 and above</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full Time	</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.5	</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>	</t>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Emory University</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>10001</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">N002	</t>
+          <t>Emory Saint Josephs</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emory Saint Josephs Hospital	</t>
+          <t>02/15/2023</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">01/15/2023	</t>
+          <t>N002</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nurse B	</t>
+          <t>99002</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">01/10/2023	</t>
+          <t>02/10/2023</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical/Surgical	</t>
+          <t>ICU</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">32	</t>
+          <t>30</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Female	</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kennesaw State University	</t>
+          <t>Georgia State</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSN	</t>
+          <t>BSN</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full Time	</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.0 - 3.49	</t>
+          <t>3.0 - 3.49</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes	</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.0	</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>	</t>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Georgia State</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>10002</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N003	</t>
+          <t>Emory Decatur</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emory Decatur Hospital	</t>
+          <t>03/01/2022</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">05/20/2022	</t>
+          <t>N003</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nurse C	</t>
+          <t>99003</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">05/15/2022	</t>
+          <t>03/01/2022</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICU	</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">24	</t>
+          <t>35</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Male	</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Georgia State University	</t>
+          <t>Kennesaw State</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADN/ASN	</t>
+          <t>BSN</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.5 - 2.99	</t>
+          <t>2.5 - 2.99</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full Time	</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
+          <t>LPN/LVN</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes	</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t xml:space="preserve">11/30/2023	</t>
+          <t>11/30/2023</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.583	</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">manager@emory.com	</t>
+          <t>Resigned</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Kennesaw State</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>10003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">N004	</t>
+          <t>Emory Midtown</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emory University Hospital Midtown	</t>
+          <t>10/01/2023</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">08/28/2022	</t>
+          <t>N004</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nurse D	</t>
+          <t>99004</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">08/04/2022	</t>
+          <t>10/01/2023</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pediatrics	</t>
+          <t>ER</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">26	</t>
+          <t>26</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Female	</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Clayton State University	</t>
+          <t>UGA</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSN	</t>
+          <t>BSN</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.0 - 3.49	</t>
+          <t>3.0 - 3.49</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full Time	</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>	</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>UGA</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>10004</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">N005	</t>
+          <t>Emory Johns Creek</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emory Saint Josephs Hospital	</t>
+          <t>05/15/2023</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">01/15/2024	</t>
+          <t>N005</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nurse E	</t>
+          <t>99005</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">01/10/2024	</t>
+          <t>05/10/2023</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oncology	</t>
+          <t>NICU</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">29	</t>
+          <t>29</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Female	</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve">University of Georgia	</t>
+          <t>Albany State</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSN	</t>
+          <t>Albany State fragment</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.5 and above	</t>
+          <t>BSN</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Part Time	</t>
+          <t>3.5 and above</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
+          <t>Full-time</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.5	</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>	</t>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Albany State University</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>10005</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">N006	</t>
+          <t>Emory University Hospital</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emory Decatur Hospital	</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">05/20/2023	</t>
+          <t>N006</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nurse F	</t>
+          <t>99006</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">05/15/2023	</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">NICU	</t>
+          <t>Med/Surg</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">31	</t>
+          <t>30</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Male	</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mercer University	</t>
+          <t>Georgia Tech</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSN	</t>
+          <t>BSN</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.0 - 2.49	</t>
+          <t>2.0 - 2.49</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full Time	</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes	</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes	</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08/15/2024	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.25	</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Personal reasons	</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hr@emory.com	</t>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Georgia Tech</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>10006</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">N007	</t>
+          <t>Emory University Hospital</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emory University Hospital Midtown	</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">08/28/2021	</t>
+          <t>N007</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nurse G	</t>
+          <t>99007</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">08/04/2021	</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emergency	</t>
+          <t>Med/Surg</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">27	</t>
+          <t>30</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Female	</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Georgia Southern University	</t>
+          <t>Georgia Tech</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSN	</t>
+          <t>BSN</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t xml:space="preserve">below 2.0	</t>
+          <t>2.0 - 2.49</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full Time	</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.0	</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>	</t>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Georgia Tech</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>10007</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">N008	</t>
+          <t>Emory University Hospital</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emory Saint Josephs Hospital	</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">01/15/2022	</t>
+          <t>N008</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nurse H	</t>
+          <t>99008</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">01/10/2022	</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cardiac	</t>
+          <t>Med/Surg</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">35	</t>
+          <t>30</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Male	</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Albany State University	</t>
+          <t>Georgia Tech</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADN/ASN	</t>
+          <t>BSN</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t xml:space="preserve">honors_gpa	</t>
+          <t>2.0 - 2.49</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full Time	</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes	</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06/30/2023	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.417	</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Better opportunity	</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hr@emory.com	</t>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Georgia Tech</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>10008</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">N009	</t>
+          <t>Emory University Hospital</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emory Decatur Hospital	</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">05/20/2024	</t>
+          <t>N009</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nurse I	</t>
+          <t>99009</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">05/15/2024	</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Telemetry	</t>
+          <t>Med/Surg</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">23	</t>
+          <t>30</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Female	</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spelman College	</t>
+          <t>Georgia Tech</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSN	</t>
+          <t>BSN</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.5 and above	</t>
+          <t>2.0 - 2.49</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full Time	</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.25	</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>	</t>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Georgia Tech</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>10009</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">N010	</t>
+          <t>Emory University Hospital</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emory University Hospital Midtown	</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">08/28/2020	</t>
+          <t>N0010</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nurse J	</t>
+          <t>990010</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">08/04/2020	</t>
+          <t>01/01/2023</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Neuro	</t>
+          <t>Med/Surg</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">40	</t>
+          <t>30</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Female	</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Howard University	</t>
+          <t>Georgia Tech</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve">BSN	</t>
+          <t>BSN</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.0 - 3.49	</t>
+          <t>2.0 - 2.49</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full Time	</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t xml:space="preserve">No	</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.5	</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>	</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>	</t>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Georgia Tech</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>100010</t>
         </is>
       </c>
     </row>

</xml_diff>